<commit_message>
Regenerate full 2026-06-03 report and improve local trigger errors
</commit_message>
<xml_diff>
--- a/docs/pension_data_combined_2026-06-03.xlsx
+++ b/docs/pension_data_combined_2026-06-03.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.12" customWidth="1" min="1" max="1"/>
@@ -454,165 +454,165 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ARTEA</t>
+          <t>ALLIANZ</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Artea pensija 2003-2009</t>
+          <t>Allianz D1 gimusiems 2003-2009 m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.2243</v>
+        <v>1.1759</v>
       </c>
       <c r="D3" t="n">
-        <v>3041679.12</v>
+        <v>2088389.39</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Artea pensija 1996-2002</t>
+          <t>Allianz S turto išsaugojimo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.318</v>
+        <v>1.1824</v>
       </c>
       <c r="D4" t="n">
-        <v>36180414.83000001</v>
+        <v>35036425.03</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Artea pensija 1989-1995</t>
+          <t>Allianz X1 gimusiems 1961–1967 m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.3011</v>
+        <v>1.453</v>
       </c>
       <c r="D5" t="n">
-        <v>126626987.28</v>
+        <v>187569033.16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Artea pensija 1982-1988</t>
+          <t>Allianz X2 gimusiems 1968–1974 m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.307</v>
+        <v>1.9705</v>
       </c>
       <c r="D6" t="n">
-        <v>234277824.21</v>
+        <v>216994358.43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Artea pensija 1975-1981</t>
+          <t>Allianz X3 gimusiems 1975–1981 m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.2845</v>
+        <v>2.2422</v>
       </c>
       <c r="D7" t="n">
-        <v>228764648.92</v>
+        <v>222595478.33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Artea pensija 1968-1974</t>
+          <t>Allianz Y1 gimusiems 1982–1988 m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.9741</v>
+        <v>2.281</v>
       </c>
       <c r="D8" t="n">
-        <v>169581995.12</v>
+        <v>180575433.92</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Artea pensija 1961-1967</t>
+          <t>Allianz Y2 gimusiems 1989–1995 m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.5562</v>
+        <v>2.2748</v>
       </c>
       <c r="D9" t="n">
-        <v>112117010.1</v>
+        <v>98552267.84999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Artea pensijų turto išsaugojimo fondas</t>
+          <t>Allianz Y3 gimusiems 1996–2002 m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.2531</v>
+        <v>2.2573</v>
       </c>
       <c r="D10" t="n">
-        <v>17442354.38</v>
+        <v>38162426.53</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GOINDEX</t>
+          <t>ARTEA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Goindex pensija 2003-2009</t>
+          <t>Artea pensija 2003-2009</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -621,16 +621,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.2047</v>
+        <v>1.2199</v>
       </c>
       <c r="D12" t="n">
-        <v>4364080.4278</v>
+        <v>3032400.46</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Goindex pensija 1996-2002</t>
+          <t>Artea pensija 1996-2002</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.5851</v>
+        <v>2.3126</v>
       </c>
       <c r="D13" t="n">
-        <v>27723696.8467</v>
+        <v>36086627.89</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Goindex pensija 1989-1995</t>
+          <t>Artea pensija 1989-1995</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -657,16 +657,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.5813</v>
+        <v>2.2965</v>
       </c>
       <c r="D14" t="n">
-        <v>50062301.9338</v>
+        <v>126369011.96</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Goindex pensija 1982-1988</t>
+          <t>Artea pensija 1982-1988</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -675,16 +675,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.5902</v>
+        <v>2.3019</v>
       </c>
       <c r="D15" t="n">
-        <v>61942699.0432</v>
+        <v>233747915.41</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Goindex pensija 1975-1981</t>
+          <t>Artea pensija 1975-1981</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.5828</v>
+        <v>2.2797</v>
       </c>
       <c r="D16" t="n">
-        <v>56576796.5224</v>
+        <v>228317318.39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Goindex pensija 1968-1974</t>
+          <t>Artea pensija 1968-1974</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -711,16 +711,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.5655</v>
+        <v>1.9706</v>
       </c>
       <c r="D17" t="n">
-        <v>37390408.0913</v>
+        <v>169272265.01</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Goindex pensija 1961-1967</t>
+          <t>Artea pensija 1961-1967</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -729,28 +729,632 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.2664</v>
+        <v>1.5531</v>
       </c>
       <c r="D18" t="n">
-        <v>10815276.2448</v>
+        <v>111776999.55</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Artea pensijų turto išsaugojimo fondas</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1.2515</v>
+      </c>
+      <c r="D19" t="n">
+        <v>17418856.93</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GOINDEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Goindex pensija 2003-2009</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1.2047</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4364080.4278</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Goindex pensija 1996-2002</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1.5851</v>
+      </c>
+      <c r="D22" t="n">
+        <v>27723696.8467</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Goindex pensija 1989-1995</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1.5813</v>
+      </c>
+      <c r="D23" t="n">
+        <v>50062301.9338</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Goindex pensija 1982-1988</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1.5902</v>
+      </c>
+      <c r="D24" t="n">
+        <v>61942699.0432</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Goindex pensija 1975-1981</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1.5828</v>
+      </c>
+      <c r="D25" t="n">
+        <v>56576796.5224</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Goindex pensija 1968-1974</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1.5655</v>
+      </c>
+      <c r="D26" t="n">
+        <v>37390408.0913</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Goindex pensija 1961-1967</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1.2664</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10815276.2448</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Goindex pensijų turto išsaugojimo fondas</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
         <v>1.0917</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D28" t="n">
         <v>1736182.5938</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LUMINOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Luminor 2003-2009 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1.1876</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3781198.35</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Luminor 1996-2002 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2.2971</v>
+      </c>
+      <c r="D31" t="n">
+        <v>22135327.78</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Luminor 1989-1995 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2.2842</v>
+      </c>
+      <c r="D32" t="n">
+        <v>61277393.09</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Luminor 1982-1988 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2.2682</v>
+      </c>
+      <c r="D33" t="n">
+        <v>117869035.56</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Luminor 1975-1981 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2.2663</v>
+      </c>
+      <c r="D34" t="n">
+        <v>127610742.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Luminor 1968-1974 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2.0625</v>
+      </c>
+      <c r="D35" t="n">
+        <v>112187068.17</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Luminor 1961-1967 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1.5807</v>
+      </c>
+      <c r="D36" t="n">
+        <v>89817396.73999999</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Luminor pensijų turto išsaugojimo fondas</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1.1707</v>
+      </c>
+      <c r="D37" t="n">
+        <v>14650943.54</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SEB pensija 2003-2009</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1.1834</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2571128</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SEB pensija 1996-2002</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2.3543</v>
+      </c>
+      <c r="D40" t="n">
+        <v>47346973</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SEB pensija 1989-1995</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.3334</v>
+      </c>
+      <c r="D41" t="n">
+        <v>155697641</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SEB pensija 1982-1988</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2.3376</v>
+      </c>
+      <c r="D42" t="n">
+        <v>378269261</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SEB pensija 1975-1981</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.3693</v>
+      </c>
+      <c r="D43" t="n">
+        <v>482315353</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SEB pensija 1968-1974</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2.0424</v>
+      </c>
+      <c r="D44" t="n">
+        <v>394304007</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SEB pensija 1961-1967</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.5559</v>
+      </c>
+      <c r="D45" t="n">
+        <v>294928845</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SEB turto išsaugojimo fondas</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.2138</v>
+      </c>
+      <c r="D46" t="n">
+        <v>58220500</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SWEDBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Pensija 2003-2009</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1.1357</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3738153.96</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Pensija 1996-2002</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2.1342</v>
+      </c>
+      <c r="D49" t="n">
+        <v>83654600.7</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Pensija 1989-1995</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2.1532</v>
+      </c>
+      <c r="D50" t="n">
+        <v>269103438.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Pensija 1982-1988</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2.171</v>
+      </c>
+      <c r="D51" t="n">
+        <v>410309971.8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Pensija 1975-1981</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2.1765</v>
+      </c>
+      <c r="D52" t="n">
+        <v>500230230.3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Pensija 1968-1974</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1.9653</v>
+      </c>
+      <c r="D53" t="n">
+        <v>467424929.9</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pensija 1961-1967</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1.5429</v>
+      </c>
+      <c r="D54" t="n">
+        <v>368313507.8</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Turto išsaugojimo pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1.2033</v>
+      </c>
+      <c r="D55" t="n">
+        <v>68446980.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>